<commit_message>
Update report: 해안면 20260318_20260325
</commit_message>
<xml_diff>
--- a/shucle_report/해안면/20260318_20260325/report_해안면_20260318_20260325.xlsx
+++ b/shucle_report/해안면/20260318_20260325/report_해안면_20260318_20260325.xlsx
@@ -514,7 +514,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>분석기간: 2026.03.18 ~ 03.25 | 비교기간: 2026.03.11 ~ 03.17 | 생성: 2026-03-26 14:48 | 차트: 78개</t>
+          <t>분석기간: 2026.03.18 ~ 03.25 | 비교기간: 2026.03.11 ~ 03.17 | 생성: 2026-03-26 15:08 | 차트: 123개</t>
         </is>
       </c>
     </row>
@@ -582,27 +582,27 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.4건</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8.5건</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+2.1건</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>+32.8%</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>⚠ 증가</t>
         </is>
       </c>
     </row>
@@ -619,27 +619,27 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5.6건</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7.7건</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+2.1건</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>+36.9%</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>⚠ 증가</t>
         </is>
       </c>
     </row>
@@ -656,27 +656,27 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.2명</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9.3명</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+3.1명</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>+50.5%</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>⚠ 증가</t>
         </is>
       </c>
     </row>
@@ -915,22 +915,22 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>93.8%</t>
+          <t>87.8%</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>91.7%</t>
+          <t>89.4%</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>-2.1%p</t>
+          <t>+1.6%p</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>-2.2%</t>
+          <t>+1.8%</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -1104,7 +1104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1126,7 +1126,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>▲ 대당 탑승객 수(일평균) (+50.5%)</t>
+          <t>▲ 실시간 호출 건수(일평균) (+32.8%)</t>
         </is>
       </c>
     </row>
@@ -1170,192 +1170,192 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>대당 탑승객 수(일평균)</t>
+          <t>실시간 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>대당 탑승객 수(평일)</t>
+          <t>이동완료 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>9.3</t>
+          <t>7.7</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>+3.1</t>
+          <t>+2.1</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>+50.5%</t>
+          <t>+36.9%</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>평일 9.3명 (51% 증가)</t>
+          <t>동반 증가 (37%)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>대당 탑승객 수(일평균)</t>
+          <t>실시간 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>대당 탑승객 수(주말)</t>
+          <t>평균 대기시간</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-0.4</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-11.7%</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>3.8→3.3분 감소</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>대당 탑승객 수(일평균)</t>
+          <t>실시간 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>동승 인원 분포(일평균)</t>
+          <t>전화 호출 비율</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>43.8%</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>33.3%</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-10.4%p</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-23.8%</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>전화 44→33%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>대당 탑승객 수(일평균)</t>
+          <t>실시간 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>실시간 호출 건수(일평균)</t>
+          <t>앱 호출 비율</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>28.1%</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>52.9%</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+24.8%p</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+88.2%</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>앱 비중 53%로 주도적</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>대당 탑승객 수(일평균)</t>
+          <t>실시간 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>운행차량 대수</t>
+          <t>현장 호출 비율</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>28.1%</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>+0.0</t>
+          <t>-14.4%p</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>-51.2%</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>1대 유지, 증차 여지 없음</t>
+          <t>현장 28→14%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>▲ 평균 우회비율 (+28.3%)</t>
+          <t>▲ 이동완료 호출 건수(일평균) (+36.9%)</t>
         </is>
       </c>
     </row>
@@ -1399,118 +1399,118 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>평균 우회비율</t>
+          <t>이동완료 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>상위 10% 우회비율</t>
+          <t>미탑승 건수(일평균)</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>+0.7</t>
+          <t>+0.1</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>+48.3%</t>
+          <t>+66.7%</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>2.1배, 우회 심화</t>
+          <t>미탑승 건수 67% 증가</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>평균 우회비율</t>
+          <t>이동완료 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>평균 이동시간</t>
+          <t>호출취소 건수(일평균)</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>-0.1</t>
+          <t>-0.0</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>-2.4%</t>
+          <t>-16.7%</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>4.2분 안정</t>
+          <t>호출취소 건수 17% 감소</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>평균 우회비율</t>
+          <t>이동완료 호출 건수(일평균)</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>동승 인원 분포(일평균)</t>
+          <t>배차실패 건수(일평균)</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-0.1</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-16.7%</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>배차실패 건수 17% 감소</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>▲ DAU (일간 활성 회원) (+66.7%)</t>
+          <t>▲ 총 탑승객 수(일평균) (+50.5%)</t>
         </is>
       </c>
     </row>
@@ -1554,194 +1554,773 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>DAU (일간 활성 회원)</t>
+          <t>총 탑승객 수(일평균)</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>WAU (주간 활성 회원)</t>
+          <t>동승 인원 분포(일평균)</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>-0.4</t>
+          <t>+3.1</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>-11.5%</t>
+          <t>+50.5%</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>3.2→2.8명 감소</t>
+          <t>동반 증가 (51%)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>DAU (일간 활성 회원)</t>
+          <t>총 탑승객 수(일평균)</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>신규 지역 회원(일평균)</t>
+          <t>고령자(60+) 호출 비율</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>61.0%</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>65.5%</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>+0.1</t>
+          <t>+4.4%p</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>+6.1%</t>
+          <t>+7.2%</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>신규 2.3명/일 (6% 증가)</t>
+          <t>고령자(60+) 비중 65%로 주도적</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>DAU (일간 활성 회원)</t>
+          <t>총 탑승객 수(일평균)</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>활성 회원 평균연령</t>
+          <t>성인(20~50대) 호출 비율</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>61.7</t>
+          <t>39.0%</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>73.0</t>
+          <t>34.5%</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>+11.3</t>
+          <t>-4.4%p</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>+18.4%</t>
+          <t>-11.3%</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>평균 73세 (18% 증가)</t>
+          <t>성인(20~50대) 39→35%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
+          <t>총 탑승객 수(일평균)</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>어린이/청소년 호출 비율</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>+0.0%p</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>변동 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>▲ 대당 탑승객 수(일평균) (+50.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>세부지표</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>비교기간</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>분석기간</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>변동값</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>변동률</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>포인트</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>대당 탑승객 수(일평균)</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>대당 탑승객 수(평일)</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>+3.1</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>+50.5%</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>평일 9.3명 (51% 증가)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>대당 탑승객 수(일평균)</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>대당 탑승객 수(주말)</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>데이터 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>대당 탑승객 수(일평균)</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>동승 인원 분포(일평균)</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>+3.1</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>+50.5%</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>동반 증가 (51%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>대당 탑승객 수(일평균)</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>실시간 호출 건수(일평균)</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>6.4</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>+2.1</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>+32.8%</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>동반 증가 (33%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>대당 탑승객 수(일평균)</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>운행차량 대수</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>+0.0</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>1대 유지, 증차 여지 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>▲ 평균 우회비율 (+28.3%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>세부지표</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>비교기간</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>분석기간</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>변동값</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>변동률</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>포인트</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>평균 우회비율</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>상위 10% 우회비율</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>+0.7</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>+48.3%</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>2.1배, 우회 심화</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>평균 우회비율</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>평균 이동시간</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>-0.1</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>-2.4%</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>4.2분 안정</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>평균 우회비율</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>동승 인원 분포(일평균)</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>+3.1</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>+50.5%</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>51% 증가, 주요 요인</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>▲ DAU (일간 활성 회원) (+66.7%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>세부지표</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>비교기간</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>분석기간</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>변동값</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>변동률</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>포인트</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
           <t>DAU (일간 활성 회원)</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>WAU (주간 활성 회원)</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>-0.4</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>-11.5%</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>3.2→2.8명 감소</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>DAU (일간 활성 회원)</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>신규 지역 회원(일평균)</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>+0.1</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>+6.1%</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>신규 2.3명/일 (6% 증가)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>DAU (일간 활성 회원)</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>활성 회원 평균연령</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>61.7</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>73.0</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>+11.3</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>+18.4%</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>평균 73세 (18% 증가)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>DAU (일간 활성 회원)</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>가호출 성공률</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>93.8%</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>87.8%</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
         <is>
           <t>89.4%</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>-4.4%p</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>-4.7%</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>+1.6%p</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>+1.8%</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
         <is>
           <t>안정 유지, 영향 제한적</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>DAU (일간 활성 회원)</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>평균 대기시간</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C44" s="7" t="inlineStr">
         <is>
           <t>3.8</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D44" s="7" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E44" s="7" t="inlineStr">
         <is>
           <t>-0.4</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F44" s="7" t="inlineStr">
         <is>
           <t>-11.7%</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="G44" s="6" t="inlineStr">
         <is>
           <t>3.8→3.3분 감소</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A11:G11"/>
+  <mergeCells count="7">
+    <mergeCell ref="A32:G32"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A11:G11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1753,7 +2332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1769,28 +2348,35 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>• 대기시간 개선: 3.8분 → 3.3분 (-12%) — 특히 03/19 상위10% 대기시간 10.2분으로 극단치 발생</t>
+          <t>• 수요 증가: 호출(+33%), 이동완료(+37%), 탑승객(+51%) 모두 상승 — 분석기간 운행 6일(03/18,03/19,03/20,03/23,03/24,03/25), 비교기간 5일</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>• 성장 지표 긍정적: DAU +67%, 누적 29명</t>
+          <t>• 이동완료율 87.5% → 90.2% (+2.7%p): 호출 8건 중 8건 완료 (호출취소 1건, 배차실패 2건)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>• 가호출 성공률 안정: 93.8% → 91.7% (-2.2%)</t>
+          <t>• 대기시간 개선: 3.8분 → 3.3분 (-12%) — 특히 03/19 상위10% 대기시간 10.2분으로 극단치 발생</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>• 공급 현황: 운행차량 1.0대, 대당 운행시간 7.1시간</t>
+          <t>• 성장 지표 긍정적: DAU +67%, 누적 29명</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>• 호출당 평균 탑승객 1.2명: 1인 이용 위주</t>
         </is>
       </c>
     </row>
@@ -2069,27 +2655,27 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+2.1</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+32.8%</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>역방향 증가 (33%)</t>
         </is>
       </c>
     </row>
@@ -2145,32 +2731,32 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>피크 시간대 이동시간</t>
+          <t>피크 시간대(15~17시) 이동시간</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.9</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-2.2</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-32.6%</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>6.9→4.6분 감소</t>
         </is>
       </c>
     </row>
@@ -2182,32 +2768,32 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>비피크 시간대 이동시간</t>
+          <t>비피크 시간대(8~10시) 이동시간</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+0.9</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+23.0%</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>3.9→4.8분 증가</t>
         </is>
       </c>
     </row>
@@ -2379,27 +2965,27 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-0.1</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-16.7%</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>배차실패 건수 17% 감소</t>
         </is>
       </c>
     </row>
@@ -2561,7 +3147,7 @@
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>▼ 가호출 성공률 (-2.2%)</t>
+          <t>▲ 가호출 성공률 (+1.8%)</t>
         </is>
       </c>
     </row>
@@ -2615,27 +3201,27 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>93.8%</t>
+          <t>87.8%</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>91.7%</t>
+          <t>89.4%</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>-2.1%p</t>
+          <t>+1.6%p</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>-2.2%</t>
+          <t>+1.8%</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>평일 92% (2% 감소)</t>
+          <t>평일 89% (2% 증가)</t>
         </is>
       </c>
     </row>
@@ -2918,27 +3504,27 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+2.1</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+32.8%</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>역방향 증가 (33%)</t>
         </is>
       </c>
     </row>

</xml_diff>